<commit_message>
feat: update example file when import product list
</commit_message>
<xml_diff>
--- a/hddt-SES/src/main/resources/static/file_product/Mau-Import-Danh-Sach_San-Pham.xlsx
+++ b/hddt-SES/src/main/resources/static/file_product/Mau-Import-Danh-Sach_San-Pham.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="25225"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SES_GROUP\12-05-2022 FILE MAU EXCEL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/11c1a6aacc2e6d99/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F586A2BF-0FDF-4CC3-949F-CC21A2A8D123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{F586A2BF-0FDF-4CC3-949F-CC21A2A8D123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F81792A-FA6A-418C-B732-DF88E1199483}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13216" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -32,18 +32,9 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
   <si>
-    <t>Mã sản phẩm</t>
-  </si>
-  <si>
-    <t>Tên sản phẩm</t>
-  </si>
-  <si>
     <t>Đơn giá</t>
   </si>
   <si>
-    <t>Đơn vị tính</t>
-  </si>
-  <si>
     <t>Cái</t>
   </si>
   <si>
@@ -77,9 +68,6 @@
     <t>Hạn sử dụng</t>
   </si>
   <si>
-    <t>Thuế suất GTGT</t>
-  </si>
-  <si>
     <t>SL00001</t>
   </si>
   <si>
@@ -90,13 +78,25 @@
   </si>
   <si>
     <t>Mã kho</t>
+  </si>
+  <si>
+    <t>Mã sản phẩm (*)</t>
+  </si>
+  <si>
+    <t>Tên sản phẩm(*)</t>
+  </si>
+  <si>
+    <t>Thuế suất GTGT(*)</t>
+  </si>
+  <si>
+    <t>Đơn vị tính (*)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -108,6 +108,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -167,7 +175,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -185,6 +193,12 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -466,97 +480,97 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" customWidth="1"/>
-    <col min="2" max="2" width="21.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="17.85546875" customWidth="1"/>
-    <col min="5" max="5" width="17.28515625" customWidth="1"/>
+    <col min="1" max="1" width="17.86328125" customWidth="1"/>
+    <col min="2" max="2" width="21.86328125" customWidth="1"/>
+    <col min="3" max="3" width="19.59765625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17.86328125" customWidth="1"/>
+    <col min="5" max="5" width="17.265625" customWidth="1"/>
     <col min="6" max="7" width="21" customWidth="1"/>
-    <col min="8" max="8" width="20.42578125" customWidth="1"/>
-    <col min="9" max="9" width="23.5703125" customWidth="1"/>
+    <col min="8" max="8" width="20.3984375" customWidth="1"/>
+    <col min="9" max="9" width="23.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="4" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:9" s="4" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>19</v>
-      </c>
       <c r="H1" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C2" s="5">
         <v>100000</v>
       </c>
       <c r="D2" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F2">
         <v>10</v>
       </c>
       <c r="H2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C3" s="5">
         <v>200000</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F3">
         <v>10</v>
       </c>
       <c r="H3" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>